<commit_message>
clean vs data, add sources
</commit_message>
<xml_diff>
--- a/data/datasets/wallis/VS_17/VS_17_leuk.xlsx
+++ b/data/datasets/wallis/VS_17/VS_17_leuk.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\data\datasets\wallis\VS_17\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E692A7A3-D74B-45F3-BF69-FBEC3A9A0397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Export" sheetId="1" r:id="rId4"/>
+    <sheet name="Export" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Grossräte 2017</t>
   </si>
@@ -155,23 +160,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -182,31 +179,38 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -496,220 +500,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:GQ50"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N50"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="80" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12" customWidth="true" style="0"/>
-    <col min="3" max="3" width="12" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12" customWidth="true" style="0"/>
-    <col min="5" max="5" width="12" customWidth="true" style="0"/>
-    <col min="6" max="6" width="12" customWidth="true" style="0"/>
-    <col min="7" max="7" width="12" customWidth="true" style="0"/>
-    <col min="8" max="8" width="12" customWidth="true" style="0"/>
-    <col min="9" max="9" width="12" customWidth="true" style="0"/>
-    <col min="10" max="10" width="12" customWidth="true" style="0"/>
-    <col min="11" max="11" width="12" customWidth="true" style="0"/>
-    <col min="12" max="12" width="12" customWidth="true" style="0"/>
-    <col min="13" max="13" width="12" customWidth="true" style="0"/>
-    <col min="14" max="14" width="12" customWidth="true" style="0"/>
-    <col min="15" max="15" width="12" customWidth="true" style="0"/>
-    <col min="16" max="16" width="12" customWidth="true" style="0"/>
-    <col min="17" max="17" width="12" customWidth="true" style="0"/>
-    <col min="18" max="18" width="12" customWidth="true" style="0"/>
-    <col min="19" max="19" width="12" customWidth="true" style="0"/>
-    <col min="20" max="20" width="12" customWidth="true" style="0"/>
-    <col min="21" max="21" width="12" customWidth="true" style="0"/>
-    <col min="22" max="22" width="12" customWidth="true" style="0"/>
-    <col min="23" max="23" width="12" customWidth="true" style="0"/>
-    <col min="24" max="24" width="12" customWidth="true" style="0"/>
-    <col min="25" max="25" width="12" customWidth="true" style="0"/>
-    <col min="26" max="26" width="12" customWidth="true" style="0"/>
-    <col min="27" max="27" width="12" customWidth="true" style="0"/>
-    <col min="28" max="28" width="12" customWidth="true" style="0"/>
-    <col min="29" max="29" width="12" customWidth="true" style="0"/>
-    <col min="30" max="30" width="12" customWidth="true" style="0"/>
-    <col min="31" max="31" width="12" customWidth="true" style="0"/>
-    <col min="32" max="32" width="12" customWidth="true" style="0"/>
-    <col min="33" max="33" width="12" customWidth="true" style="0"/>
-    <col min="34" max="34" width="12" customWidth="true" style="0"/>
-    <col min="35" max="35" width="12" customWidth="true" style="0"/>
-    <col min="36" max="36" width="12" customWidth="true" style="0"/>
-    <col min="37" max="37" width="12" customWidth="true" style="0"/>
-    <col min="38" max="38" width="12" customWidth="true" style="0"/>
-    <col min="39" max="39" width="12" customWidth="true" style="0"/>
-    <col min="40" max="40" width="12" customWidth="true" style="0"/>
-    <col min="41" max="41" width="12" customWidth="true" style="0"/>
-    <col min="42" max="42" width="12" customWidth="true" style="0"/>
-    <col min="43" max="43" width="12" customWidth="true" style="0"/>
-    <col min="44" max="44" width="12" customWidth="true" style="0"/>
-    <col min="45" max="45" width="12" customWidth="true" style="0"/>
-    <col min="46" max="46" width="12" customWidth="true" style="0"/>
-    <col min="47" max="47" width="12" customWidth="true" style="0"/>
-    <col min="48" max="48" width="12" customWidth="true" style="0"/>
-    <col min="49" max="49" width="12" customWidth="true" style="0"/>
-    <col min="50" max="50" width="12" customWidth="true" style="0"/>
-    <col min="51" max="51" width="12" customWidth="true" style="0"/>
-    <col min="52" max="52" width="12" customWidth="true" style="0"/>
-    <col min="53" max="53" width="12" customWidth="true" style="0"/>
-    <col min="54" max="54" width="12" customWidth="true" style="0"/>
-    <col min="55" max="55" width="12" customWidth="true" style="0"/>
-    <col min="56" max="56" width="12" customWidth="true" style="0"/>
-    <col min="57" max="57" width="12" customWidth="true" style="0"/>
-    <col min="58" max="58" width="12" customWidth="true" style="0"/>
-    <col min="59" max="59" width="12" customWidth="true" style="0"/>
-    <col min="60" max="60" width="12" customWidth="true" style="0"/>
-    <col min="61" max="61" width="12" customWidth="true" style="0"/>
-    <col min="62" max="62" width="12" customWidth="true" style="0"/>
-    <col min="63" max="63" width="12" customWidth="true" style="0"/>
-    <col min="64" max="64" width="12" customWidth="true" style="0"/>
-    <col min="65" max="65" width="12" customWidth="true" style="0"/>
-    <col min="66" max="66" width="12" customWidth="true" style="0"/>
-    <col min="67" max="67" width="12" customWidth="true" style="0"/>
-    <col min="68" max="68" width="12" customWidth="true" style="0"/>
-    <col min="69" max="69" width="12" customWidth="true" style="0"/>
-    <col min="70" max="70" width="12" customWidth="true" style="0"/>
-    <col min="71" max="71" width="12" customWidth="true" style="0"/>
-    <col min="72" max="72" width="12" customWidth="true" style="0"/>
-    <col min="73" max="73" width="12" customWidth="true" style="0"/>
-    <col min="74" max="74" width="12" customWidth="true" style="0"/>
-    <col min="75" max="75" width="12" customWidth="true" style="0"/>
-    <col min="76" max="76" width="12" customWidth="true" style="0"/>
-    <col min="77" max="77" width="12" customWidth="true" style="0"/>
-    <col min="78" max="78" width="12" customWidth="true" style="0"/>
-    <col min="79" max="79" width="12" customWidth="true" style="0"/>
-    <col min="80" max="80" width="12" customWidth="true" style="0"/>
-    <col min="81" max="81" width="12" customWidth="true" style="0"/>
-    <col min="82" max="82" width="12" customWidth="true" style="0"/>
-    <col min="83" max="83" width="12" customWidth="true" style="0"/>
-    <col min="84" max="84" width="12" customWidth="true" style="0"/>
-    <col min="85" max="85" width="12" customWidth="true" style="0"/>
-    <col min="86" max="86" width="12" customWidth="true" style="0"/>
-    <col min="87" max="87" width="12" customWidth="true" style="0"/>
-    <col min="88" max="88" width="12" customWidth="true" style="0"/>
-    <col min="89" max="89" width="12" customWidth="true" style="0"/>
-    <col min="90" max="90" width="12" customWidth="true" style="0"/>
-    <col min="91" max="91" width="12" customWidth="true" style="0"/>
-    <col min="92" max="92" width="12" customWidth="true" style="0"/>
-    <col min="93" max="93" width="12" customWidth="true" style="0"/>
-    <col min="94" max="94" width="12" customWidth="true" style="0"/>
-    <col min="95" max="95" width="12" customWidth="true" style="0"/>
-    <col min="96" max="96" width="12" customWidth="true" style="0"/>
-    <col min="97" max="97" width="12" customWidth="true" style="0"/>
-    <col min="98" max="98" width="12" customWidth="true" style="0"/>
-    <col min="99" max="99" width="12" customWidth="true" style="0"/>
-    <col min="100" max="100" width="12" customWidth="true" style="0"/>
-    <col min="101" max="101" width="12" customWidth="true" style="0"/>
-    <col min="102" max="102" width="12" customWidth="true" style="0"/>
-    <col min="103" max="103" width="12" customWidth="true" style="0"/>
-    <col min="104" max="104" width="12" customWidth="true" style="0"/>
-    <col min="105" max="105" width="12" customWidth="true" style="0"/>
-    <col min="106" max="106" width="12" customWidth="true" style="0"/>
-    <col min="107" max="107" width="12" customWidth="true" style="0"/>
-    <col min="108" max="108" width="12" customWidth="true" style="0"/>
-    <col min="109" max="109" width="12" customWidth="true" style="0"/>
-    <col min="110" max="110" width="12" customWidth="true" style="0"/>
-    <col min="111" max="111" width="12" customWidth="true" style="0"/>
-    <col min="112" max="112" width="12" customWidth="true" style="0"/>
-    <col min="113" max="113" width="12" customWidth="true" style="0"/>
-    <col min="114" max="114" width="12" customWidth="true" style="0"/>
-    <col min="115" max="115" width="12" customWidth="true" style="0"/>
-    <col min="116" max="116" width="12" customWidth="true" style="0"/>
-    <col min="117" max="117" width="12" customWidth="true" style="0"/>
-    <col min="118" max="118" width="12" customWidth="true" style="0"/>
-    <col min="119" max="119" width="12" customWidth="true" style="0"/>
-    <col min="120" max="120" width="12" customWidth="true" style="0"/>
-    <col min="121" max="121" width="12" customWidth="true" style="0"/>
-    <col min="122" max="122" width="12" customWidth="true" style="0"/>
-    <col min="123" max="123" width="12" customWidth="true" style="0"/>
-    <col min="124" max="124" width="12" customWidth="true" style="0"/>
-    <col min="125" max="125" width="12" customWidth="true" style="0"/>
-    <col min="126" max="126" width="12" customWidth="true" style="0"/>
-    <col min="127" max="127" width="12" customWidth="true" style="0"/>
-    <col min="128" max="128" width="12" customWidth="true" style="0"/>
-    <col min="129" max="129" width="12" customWidth="true" style="0"/>
-    <col min="130" max="130" width="12" customWidth="true" style="0"/>
-    <col min="131" max="131" width="12" customWidth="true" style="0"/>
-    <col min="132" max="132" width="12" customWidth="true" style="0"/>
-    <col min="133" max="133" width="12" customWidth="true" style="0"/>
-    <col min="134" max="134" width="12" customWidth="true" style="0"/>
-    <col min="135" max="135" width="12" customWidth="true" style="0"/>
-    <col min="136" max="136" width="12" customWidth="true" style="0"/>
-    <col min="137" max="137" width="12" customWidth="true" style="0"/>
-    <col min="138" max="138" width="12" customWidth="true" style="0"/>
-    <col min="139" max="139" width="12" customWidth="true" style="0"/>
-    <col min="140" max="140" width="12" customWidth="true" style="0"/>
-    <col min="141" max="141" width="12" customWidth="true" style="0"/>
-    <col min="142" max="142" width="12" customWidth="true" style="0"/>
-    <col min="143" max="143" width="12" customWidth="true" style="0"/>
-    <col min="144" max="144" width="12" customWidth="true" style="0"/>
-    <col min="145" max="145" width="12" customWidth="true" style="0"/>
-    <col min="146" max="146" width="12" customWidth="true" style="0"/>
-    <col min="147" max="147" width="12" customWidth="true" style="0"/>
-    <col min="148" max="148" width="12" customWidth="true" style="0"/>
-    <col min="149" max="149" width="12" customWidth="true" style="0"/>
-    <col min="150" max="150" width="12" customWidth="true" style="0"/>
-    <col min="151" max="151" width="12" customWidth="true" style="0"/>
-    <col min="152" max="152" width="12" customWidth="true" style="0"/>
-    <col min="153" max="153" width="12" customWidth="true" style="0"/>
-    <col min="154" max="154" width="12" customWidth="true" style="0"/>
-    <col min="155" max="155" width="12" customWidth="true" style="0"/>
-    <col min="156" max="156" width="12" customWidth="true" style="0"/>
-    <col min="157" max="157" width="12" customWidth="true" style="0"/>
-    <col min="158" max="158" width="12" customWidth="true" style="0"/>
-    <col min="159" max="159" width="12" customWidth="true" style="0"/>
-    <col min="160" max="160" width="12" customWidth="true" style="0"/>
-    <col min="161" max="161" width="12" customWidth="true" style="0"/>
-    <col min="162" max="162" width="12" customWidth="true" style="0"/>
-    <col min="163" max="163" width="12" customWidth="true" style="0"/>
-    <col min="164" max="164" width="12" customWidth="true" style="0"/>
-    <col min="165" max="165" width="12" customWidth="true" style="0"/>
-    <col min="166" max="166" width="12" customWidth="true" style="0"/>
-    <col min="167" max="167" width="12" customWidth="true" style="0"/>
-    <col min="168" max="168" width="12" customWidth="true" style="0"/>
-    <col min="169" max="169" width="12" customWidth="true" style="0"/>
-    <col min="170" max="170" width="12" customWidth="true" style="0"/>
-    <col min="171" max="171" width="12" customWidth="true" style="0"/>
-    <col min="172" max="172" width="12" customWidth="true" style="0"/>
-    <col min="173" max="173" width="12" customWidth="true" style="0"/>
-    <col min="174" max="174" width="12" customWidth="true" style="0"/>
-    <col min="175" max="175" width="12" customWidth="true" style="0"/>
-    <col min="176" max="176" width="12" customWidth="true" style="0"/>
-    <col min="177" max="177" width="12" customWidth="true" style="0"/>
-    <col min="178" max="178" width="12" customWidth="true" style="0"/>
-    <col min="179" max="179" width="12" customWidth="true" style="0"/>
-    <col min="180" max="180" width="12" customWidth="true" style="0"/>
-    <col min="181" max="181" width="12" customWidth="true" style="0"/>
-    <col min="182" max="182" width="12" customWidth="true" style="0"/>
-    <col min="183" max="183" width="12" customWidth="true" style="0"/>
-    <col min="184" max="184" width="12" customWidth="true" style="0"/>
-    <col min="185" max="185" width="12" customWidth="true" style="0"/>
-    <col min="186" max="186" width="12" customWidth="true" style="0"/>
-    <col min="187" max="187" width="12" customWidth="true" style="0"/>
-    <col min="188" max="188" width="12" customWidth="true" style="0"/>
-    <col min="189" max="189" width="12" customWidth="true" style="0"/>
-    <col min="190" max="190" width="12" customWidth="true" style="0"/>
-    <col min="191" max="191" width="12" customWidth="true" style="0"/>
-    <col min="192" max="192" width="12" customWidth="true" style="0"/>
-    <col min="193" max="193" width="12" customWidth="true" style="0"/>
-    <col min="194" max="194" width="12" customWidth="true" style="0"/>
-    <col min="195" max="195" width="12" customWidth="true" style="0"/>
-    <col min="196" max="196" width="12" customWidth="true" style="0"/>
-    <col min="197" max="197" width="12" customWidth="true" style="0"/>
-    <col min="198" max="198" width="12" customWidth="true" style="0"/>
-    <col min="199" max="199" width="12" customWidth="true" style="0"/>
+    <col min="1" max="1" width="80" customWidth="1"/>
+    <col min="2" max="199" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:199">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:199">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -750,7 +554,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:199">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -794,7 +598,7 @@
         <v>8904</v>
       </c>
     </row>
-    <row r="6" spans="1:199">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -838,7 +642,7 @@
         <v>6364</v>
       </c>
     </row>
-    <row r="7" spans="1:199">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -882,7 +686,7 @@
         <v>6160</v>
       </c>
     </row>
-    <row r="8" spans="1:199">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -926,7 +730,7 @@
         <v>2185</v>
       </c>
     </row>
-    <row r="9" spans="1:199">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -970,7 +774,7 @@
         <v>3975</v>
       </c>
     </row>
-    <row r="10" spans="1:199">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1014,7 +818,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="11" spans="1:199">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1058,7 +862,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:199">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1102,7 +906,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:199">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1146,7 +950,7 @@
         <v>6169</v>
       </c>
     </row>
-    <row r="14" spans="1:199">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1190,7 +994,7 @@
         <v>71.47</v>
       </c>
     </row>
-    <row r="16" spans="1:199">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -1234,7 +1038,7 @@
         <v>9807</v>
       </c>
     </row>
-    <row r="17" spans="1:199">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -1278,7 +1082,7 @@
         <v>10571</v>
       </c>
     </row>
-    <row r="18" spans="1:199">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -1322,7 +1126,7 @@
         <v>4532</v>
       </c>
     </row>
-    <row r="19" spans="1:199">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -1366,7 +1170,7 @@
         <v>4269</v>
       </c>
     </row>
-    <row r="20" spans="1:199">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -1410,7 +1214,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="21" spans="1:199">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1454,12 +1258,12 @@
         <v>897</v>
       </c>
     </row>
-    <row r="23" spans="1:199">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:199">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1503,7 +1307,7 @@
         <v>1931</v>
       </c>
     </row>
-    <row r="25" spans="1:199">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1547,7 +1351,7 @@
         <v>1985</v>
       </c>
     </row>
-    <row r="26" spans="1:199">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -1591,7 +1395,7 @@
         <v>2058</v>
       </c>
     </row>
-    <row r="27" spans="1:199">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1635,7 +1439,7 @@
         <v>1752</v>
       </c>
     </row>
-    <row r="28" spans="1:199">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -1679,12 +1483,12 @@
         <v>2081</v>
       </c>
     </row>
-    <row r="30" spans="1:199">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:199">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1728,7 +1532,7 @@
         <v>2062</v>
       </c>
     </row>
-    <row r="32" spans="1:199">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1772,7 +1576,7 @@
         <v>2634</v>
       </c>
     </row>
-    <row r="33" spans="1:199">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1816,7 +1620,7 @@
         <v>2116</v>
       </c>
     </row>
-    <row r="34" spans="1:199">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -1860,12 +1664,12 @@
         <v>3759</v>
       </c>
     </row>
-    <row r="36" spans="1:199">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:199">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1909,7 +1713,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="38" spans="1:199">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1953,7 +1757,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="39" spans="1:199">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -1997,7 +1801,7 @@
         <v>1136</v>
       </c>
     </row>
-    <row r="40" spans="1:199">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -2041,12 +1845,12 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="42" spans="1:199">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:199">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -2090,7 +1894,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="44" spans="1:199">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -2134,7 +1938,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="45" spans="1:199">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -2178,7 +1982,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="46" spans="1:199">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>34</v>
       </c>
@@ -2222,12 +2026,12 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="48" spans="1:199">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="1:199">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>44</v>
       </c>
@@ -2271,7 +2075,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="50" spans="1:199">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>34</v>
       </c>
@@ -2316,17 +2120,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>